<commit_message>
feat(equip): 普通装备图标同步(zhuangbei), 道具表保留 itemType=4 装备行
</commit_message>
<xml_diff>
--- a/data-sources/道具表.xlsx
+++ b/data-sources/道具表.xlsx
@@ -582,7 +582,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AJ97"/>
+  <dimension ref="A1:AJ138"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -11254,9 +11254,4519 @@
         <v>0</v>
       </c>
     </row>
+    <row r="98">
+      <c r="A98">
+        <v>1100101</v>
+      </c>
+      <c r="B98" t="str">
+        <v>物理法杖</v>
+      </c>
+      <c r="C98" t="str">
+        <v/>
+      </c>
+      <c r="D98" t="str">
+        <v/>
+      </c>
+      <c r="E98" t="str">
+        <v>1</v>
+      </c>
+      <c r="F98" t="str">
+        <v>物理法杖</v>
+      </c>
+      <c r="G98" t="str">
+        <v>zhuangbei/101/109</v>
+      </c>
+      <c r="H98" t="str">
+        <v>zhuangbei/101/109_big</v>
+      </c>
+      <c r="I98" t="str">
+        <v/>
+      </c>
+      <c r="J98" t="str">
+        <v/>
+      </c>
+      <c r="K98" t="str">
+        <v/>
+      </c>
+      <c r="L98" t="str">
+        <v/>
+      </c>
+      <c r="M98">
+        <v>4</v>
+      </c>
+      <c r="N98" t="str">
+        <v/>
+      </c>
+      <c r="O98" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P98">
+        <v>1</v>
+      </c>
+      <c r="Q98" t="str">
+        <v/>
+      </c>
+      <c r="R98">
+        <v>1</v>
+      </c>
+      <c r="S98" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T98" t="str">
+        <v/>
+      </c>
+      <c r="U98">
+        <v>9999</v>
+      </c>
+      <c r="V98">
+        <v>1</v>
+      </c>
+      <c r="W98">
+        <v>0.5</v>
+      </c>
+      <c r="X98" t="str">
+        <v/>
+      </c>
+      <c r="Y98" t="str">
+        <v/>
+      </c>
+      <c r="Z98">
+        <v>-1</v>
+      </c>
+      <c r="AA98" t="str">
+        <v>dropbar/icon_type_1</v>
+      </c>
+      <c r="AB98" t="str">
+        <v/>
+      </c>
+      <c r="AC98" t="str">
+        <v/>
+      </c>
+      <c r="AD98">
+        <v>0</v>
+      </c>
+      <c r="AE98" t="str">
+        <v/>
+      </c>
+      <c r="AF98" t="str">
+        <v/>
+      </c>
+      <c r="AG98" t="str">
+        <v/>
+      </c>
+      <c r="AH98" t="str">
+        <v/>
+      </c>
+      <c r="AI98" t="str">
+        <v/>
+      </c>
+      <c r="AJ98">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99">
+        <v>1100102</v>
+      </c>
+      <c r="B99" t="str">
+        <v>火焰法杖</v>
+      </c>
+      <c r="C99" t="str">
+        <v/>
+      </c>
+      <c r="D99" t="str">
+        <v/>
+      </c>
+      <c r="E99" t="str">
+        <v>1</v>
+      </c>
+      <c r="F99" t="str">
+        <v>火焰法杖</v>
+      </c>
+      <c r="G99" t="str">
+        <v>zhuangbei/108/109</v>
+      </c>
+      <c r="H99" t="str">
+        <v>zhuangbei/108/109_big</v>
+      </c>
+      <c r="I99" t="str">
+        <v/>
+      </c>
+      <c r="J99" t="str">
+        <v/>
+      </c>
+      <c r="K99" t="str">
+        <v/>
+      </c>
+      <c r="L99" t="str">
+        <v/>
+      </c>
+      <c r="M99">
+        <v>4</v>
+      </c>
+      <c r="N99" t="str">
+        <v/>
+      </c>
+      <c r="O99" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P99">
+        <v>1</v>
+      </c>
+      <c r="Q99" t="str">
+        <v/>
+      </c>
+      <c r="R99">
+        <v>1</v>
+      </c>
+      <c r="S99" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T99" t="str">
+        <v/>
+      </c>
+      <c r="U99">
+        <v>9999</v>
+      </c>
+      <c r="V99">
+        <v>1</v>
+      </c>
+      <c r="W99">
+        <v>0.5</v>
+      </c>
+      <c r="X99" t="str">
+        <v/>
+      </c>
+      <c r="Y99" t="str">
+        <v/>
+      </c>
+      <c r="Z99">
+        <v>-1</v>
+      </c>
+      <c r="AA99" t="str">
+        <v>dropbar/icon_type_1</v>
+      </c>
+      <c r="AB99" t="str">
+        <v/>
+      </c>
+      <c r="AC99" t="str">
+        <v/>
+      </c>
+      <c r="AD99">
+        <v>0</v>
+      </c>
+      <c r="AE99" t="str">
+        <v/>
+      </c>
+      <c r="AF99" t="str">
+        <v/>
+      </c>
+      <c r="AG99" t="str">
+        <v/>
+      </c>
+      <c r="AH99" t="str">
+        <v/>
+      </c>
+      <c r="AI99" t="str">
+        <v/>
+      </c>
+      <c r="AJ99">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100">
+        <v>1100103</v>
+      </c>
+      <c r="B100" t="str">
+        <v>冰霜法杖</v>
+      </c>
+      <c r="C100" t="str">
+        <v/>
+      </c>
+      <c r="D100" t="str">
+        <v/>
+      </c>
+      <c r="E100" t="str">
+        <v>1</v>
+      </c>
+      <c r="F100" t="str">
+        <v>冰霜法杖</v>
+      </c>
+      <c r="G100" t="str">
+        <v>zhuangbei/106/109</v>
+      </c>
+      <c r="H100" t="str">
+        <v>zhuangbei/106/109_big</v>
+      </c>
+      <c r="I100" t="str">
+        <v/>
+      </c>
+      <c r="J100" t="str">
+        <v/>
+      </c>
+      <c r="K100" t="str">
+        <v/>
+      </c>
+      <c r="L100" t="str">
+        <v/>
+      </c>
+      <c r="M100">
+        <v>4</v>
+      </c>
+      <c r="N100" t="str">
+        <v/>
+      </c>
+      <c r="O100" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P100">
+        <v>1</v>
+      </c>
+      <c r="Q100" t="str">
+        <v/>
+      </c>
+      <c r="R100">
+        <v>1</v>
+      </c>
+      <c r="S100" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T100" t="str">
+        <v/>
+      </c>
+      <c r="U100">
+        <v>9999</v>
+      </c>
+      <c r="V100">
+        <v>1</v>
+      </c>
+      <c r="W100">
+        <v>0.5</v>
+      </c>
+      <c r="X100" t="str">
+        <v/>
+      </c>
+      <c r="Y100" t="str">
+        <v/>
+      </c>
+      <c r="Z100">
+        <v>-1</v>
+      </c>
+      <c r="AA100" t="str">
+        <v>dropbar/icon_type_1</v>
+      </c>
+      <c r="AB100" t="str">
+        <v/>
+      </c>
+      <c r="AC100" t="str">
+        <v/>
+      </c>
+      <c r="AD100">
+        <v>0</v>
+      </c>
+      <c r="AE100" t="str">
+        <v/>
+      </c>
+      <c r="AF100" t="str">
+        <v/>
+      </c>
+      <c r="AG100" t="str">
+        <v/>
+      </c>
+      <c r="AH100" t="str">
+        <v/>
+      </c>
+      <c r="AI100" t="str">
+        <v/>
+      </c>
+      <c r="AJ100">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101">
+        <v>1100104</v>
+      </c>
+      <c r="B101" t="str">
+        <v>闪电法杖</v>
+      </c>
+      <c r="C101" t="str">
+        <v/>
+      </c>
+      <c r="D101" t="str">
+        <v/>
+      </c>
+      <c r="E101" t="str">
+        <v>1</v>
+      </c>
+      <c r="F101" t="str">
+        <v>闪电法杖</v>
+      </c>
+      <c r="G101" t="str">
+        <v>zhuangbei/105/109</v>
+      </c>
+      <c r="H101" t="str">
+        <v>zhuangbei/105/109_big</v>
+      </c>
+      <c r="I101" t="str">
+        <v/>
+      </c>
+      <c r="J101" t="str">
+        <v/>
+      </c>
+      <c r="K101" t="str">
+        <v/>
+      </c>
+      <c r="L101" t="str">
+        <v/>
+      </c>
+      <c r="M101">
+        <v>4</v>
+      </c>
+      <c r="N101" t="str">
+        <v/>
+      </c>
+      <c r="O101" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P101">
+        <v>1</v>
+      </c>
+      <c r="Q101" t="str">
+        <v/>
+      </c>
+      <c r="R101">
+        <v>1</v>
+      </c>
+      <c r="S101" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T101" t="str">
+        <v/>
+      </c>
+      <c r="U101">
+        <v>9999</v>
+      </c>
+      <c r="V101">
+        <v>1</v>
+      </c>
+      <c r="W101">
+        <v>0.5</v>
+      </c>
+      <c r="X101" t="str">
+        <v/>
+      </c>
+      <c r="Y101" t="str">
+        <v/>
+      </c>
+      <c r="Z101">
+        <v>-1</v>
+      </c>
+      <c r="AA101" t="str">
+        <v>dropbar/icon_type_1</v>
+      </c>
+      <c r="AB101" t="str">
+        <v/>
+      </c>
+      <c r="AC101" t="str">
+        <v/>
+      </c>
+      <c r="AD101">
+        <v>0</v>
+      </c>
+      <c r="AE101" t="str">
+        <v/>
+      </c>
+      <c r="AF101" t="str">
+        <v/>
+      </c>
+      <c r="AG101" t="str">
+        <v/>
+      </c>
+      <c r="AH101" t="str">
+        <v/>
+      </c>
+      <c r="AI101" t="str">
+        <v/>
+      </c>
+      <c r="AJ101">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102">
+        <v>1100105</v>
+      </c>
+      <c r="B102" t="str">
+        <v>混沌法杖</v>
+      </c>
+      <c r="C102" t="str">
+        <v/>
+      </c>
+      <c r="D102" t="str">
+        <v/>
+      </c>
+      <c r="E102" t="str">
+        <v>1</v>
+      </c>
+      <c r="F102" t="str">
+        <v>混沌法杖</v>
+      </c>
+      <c r="G102" t="str">
+        <v>zhuangbei/107/109</v>
+      </c>
+      <c r="H102" t="str">
+        <v>zhuangbei/107/109_big</v>
+      </c>
+      <c r="I102" t="str">
+        <v/>
+      </c>
+      <c r="J102" t="str">
+        <v/>
+      </c>
+      <c r="K102" t="str">
+        <v/>
+      </c>
+      <c r="L102" t="str">
+        <v/>
+      </c>
+      <c r="M102">
+        <v>4</v>
+      </c>
+      <c r="N102" t="str">
+        <v/>
+      </c>
+      <c r="O102" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P102">
+        <v>1</v>
+      </c>
+      <c r="Q102" t="str">
+        <v/>
+      </c>
+      <c r="R102">
+        <v>1</v>
+      </c>
+      <c r="S102" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T102" t="str">
+        <v/>
+      </c>
+      <c r="U102">
+        <v>9999</v>
+      </c>
+      <c r="V102">
+        <v>1</v>
+      </c>
+      <c r="W102">
+        <v>0.5</v>
+      </c>
+      <c r="X102" t="str">
+        <v/>
+      </c>
+      <c r="Y102" t="str">
+        <v/>
+      </c>
+      <c r="Z102">
+        <v>-1</v>
+      </c>
+      <c r="AA102" t="str">
+        <v>dropbar/icon_type_1</v>
+      </c>
+      <c r="AB102" t="str">
+        <v/>
+      </c>
+      <c r="AC102" t="str">
+        <v/>
+      </c>
+      <c r="AD102">
+        <v>0</v>
+      </c>
+      <c r="AE102" t="str">
+        <v/>
+      </c>
+      <c r="AF102" t="str">
+        <v/>
+      </c>
+      <c r="AG102" t="str">
+        <v/>
+      </c>
+      <c r="AH102" t="str">
+        <v/>
+      </c>
+      <c r="AI102" t="str">
+        <v/>
+      </c>
+      <c r="AJ102">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103">
+        <v>1100201</v>
+      </c>
+      <c r="B103" t="str">
+        <v>物理长剑</v>
+      </c>
+      <c r="C103" t="str">
+        <v/>
+      </c>
+      <c r="D103" t="str">
+        <v/>
+      </c>
+      <c r="E103" t="str">
+        <v>1</v>
+      </c>
+      <c r="F103" t="str">
+        <v>物理长剑</v>
+      </c>
+      <c r="G103" t="str">
+        <v>zhuangbei/103/106</v>
+      </c>
+      <c r="H103" t="str">
+        <v>zhuangbei/103/106_big</v>
+      </c>
+      <c r="I103" t="str">
+        <v/>
+      </c>
+      <c r="J103" t="str">
+        <v/>
+      </c>
+      <c r="K103" t="str">
+        <v/>
+      </c>
+      <c r="L103" t="str">
+        <v/>
+      </c>
+      <c r="M103">
+        <v>4</v>
+      </c>
+      <c r="N103" t="str">
+        <v/>
+      </c>
+      <c r="O103" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P103">
+        <v>1</v>
+      </c>
+      <c r="Q103" t="str">
+        <v/>
+      </c>
+      <c r="R103">
+        <v>1</v>
+      </c>
+      <c r="S103" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T103" t="str">
+        <v/>
+      </c>
+      <c r="U103">
+        <v>9999</v>
+      </c>
+      <c r="V103">
+        <v>1</v>
+      </c>
+      <c r="W103">
+        <v>0.5</v>
+      </c>
+      <c r="X103" t="str">
+        <v/>
+      </c>
+      <c r="Y103" t="str">
+        <v/>
+      </c>
+      <c r="Z103">
+        <v>-1</v>
+      </c>
+      <c r="AA103" t="str">
+        <v>dropbar/icon_type_1</v>
+      </c>
+      <c r="AB103" t="str">
+        <v/>
+      </c>
+      <c r="AC103" t="str">
+        <v/>
+      </c>
+      <c r="AD103">
+        <v>0</v>
+      </c>
+      <c r="AE103" t="str">
+        <v/>
+      </c>
+      <c r="AF103" t="str">
+        <v/>
+      </c>
+      <c r="AG103" t="str">
+        <v/>
+      </c>
+      <c r="AH103" t="str">
+        <v/>
+      </c>
+      <c r="AI103" t="str">
+        <v/>
+      </c>
+      <c r="AJ103">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104">
+        <v>1100202</v>
+      </c>
+      <c r="B104" t="str">
+        <v>火焰长剑</v>
+      </c>
+      <c r="C104" t="str">
+        <v/>
+      </c>
+      <c r="D104" t="str">
+        <v/>
+      </c>
+      <c r="E104" t="str">
+        <v>1</v>
+      </c>
+      <c r="F104" t="str">
+        <v>火焰长剑</v>
+      </c>
+      <c r="G104" t="str">
+        <v>zhuangbei/108/106</v>
+      </c>
+      <c r="H104" t="str">
+        <v>zhuangbei/108/106_big</v>
+      </c>
+      <c r="I104" t="str">
+        <v/>
+      </c>
+      <c r="J104" t="str">
+        <v/>
+      </c>
+      <c r="K104" t="str">
+        <v/>
+      </c>
+      <c r="L104" t="str">
+        <v/>
+      </c>
+      <c r="M104">
+        <v>4</v>
+      </c>
+      <c r="N104" t="str">
+        <v/>
+      </c>
+      <c r="O104" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P104">
+        <v>1</v>
+      </c>
+      <c r="Q104" t="str">
+        <v/>
+      </c>
+      <c r="R104">
+        <v>1</v>
+      </c>
+      <c r="S104" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T104" t="str">
+        <v/>
+      </c>
+      <c r="U104">
+        <v>9999</v>
+      </c>
+      <c r="V104">
+        <v>1</v>
+      </c>
+      <c r="W104">
+        <v>0.5</v>
+      </c>
+      <c r="X104" t="str">
+        <v/>
+      </c>
+      <c r="Y104" t="str">
+        <v/>
+      </c>
+      <c r="Z104">
+        <v>-1</v>
+      </c>
+      <c r="AA104" t="str">
+        <v>dropbar/icon_type_1</v>
+      </c>
+      <c r="AB104" t="str">
+        <v/>
+      </c>
+      <c r="AC104" t="str">
+        <v/>
+      </c>
+      <c r="AD104">
+        <v>0</v>
+      </c>
+      <c r="AE104" t="str">
+        <v/>
+      </c>
+      <c r="AF104" t="str">
+        <v/>
+      </c>
+      <c r="AG104" t="str">
+        <v/>
+      </c>
+      <c r="AH104" t="str">
+        <v/>
+      </c>
+      <c r="AI104" t="str">
+        <v/>
+      </c>
+      <c r="AJ104">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105">
+        <v>1100203</v>
+      </c>
+      <c r="B105" t="str">
+        <v>冰霜长剑</v>
+      </c>
+      <c r="C105" t="str">
+        <v/>
+      </c>
+      <c r="D105" t="str">
+        <v/>
+      </c>
+      <c r="E105" t="str">
+        <v>1</v>
+      </c>
+      <c r="F105" t="str">
+        <v>冰霜长剑</v>
+      </c>
+      <c r="G105" t="str">
+        <v>zhuangbei/106/106</v>
+      </c>
+      <c r="H105" t="str">
+        <v>zhuangbei/106/106_big</v>
+      </c>
+      <c r="I105" t="str">
+        <v/>
+      </c>
+      <c r="J105" t="str">
+        <v/>
+      </c>
+      <c r="K105" t="str">
+        <v/>
+      </c>
+      <c r="L105" t="str">
+        <v/>
+      </c>
+      <c r="M105">
+        <v>4</v>
+      </c>
+      <c r="N105" t="str">
+        <v/>
+      </c>
+      <c r="O105" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P105">
+        <v>1</v>
+      </c>
+      <c r="Q105" t="str">
+        <v/>
+      </c>
+      <c r="R105">
+        <v>1</v>
+      </c>
+      <c r="S105" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T105" t="str">
+        <v/>
+      </c>
+      <c r="U105">
+        <v>9999</v>
+      </c>
+      <c r="V105">
+        <v>1</v>
+      </c>
+      <c r="W105">
+        <v>0.5</v>
+      </c>
+      <c r="X105" t="str">
+        <v/>
+      </c>
+      <c r="Y105" t="str">
+        <v/>
+      </c>
+      <c r="Z105">
+        <v>-1</v>
+      </c>
+      <c r="AA105" t="str">
+        <v>dropbar/icon_type_1</v>
+      </c>
+      <c r="AB105" t="str">
+        <v/>
+      </c>
+      <c r="AC105" t="str">
+        <v/>
+      </c>
+      <c r="AD105">
+        <v>0</v>
+      </c>
+      <c r="AE105" t="str">
+        <v/>
+      </c>
+      <c r="AF105" t="str">
+        <v/>
+      </c>
+      <c r="AG105" t="str">
+        <v/>
+      </c>
+      <c r="AH105" t="str">
+        <v/>
+      </c>
+      <c r="AI105" t="str">
+        <v/>
+      </c>
+      <c r="AJ105">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106">
+        <v>1100204</v>
+      </c>
+      <c r="B106" t="str">
+        <v>闪电长剑</v>
+      </c>
+      <c r="C106" t="str">
+        <v/>
+      </c>
+      <c r="D106" t="str">
+        <v/>
+      </c>
+      <c r="E106" t="str">
+        <v>1</v>
+      </c>
+      <c r="F106" t="str">
+        <v>闪电长剑</v>
+      </c>
+      <c r="G106" t="str">
+        <v>zhuangbei/105/106</v>
+      </c>
+      <c r="H106" t="str">
+        <v>zhuangbei/105/106_big</v>
+      </c>
+      <c r="I106" t="str">
+        <v/>
+      </c>
+      <c r="J106" t="str">
+        <v/>
+      </c>
+      <c r="K106" t="str">
+        <v/>
+      </c>
+      <c r="L106" t="str">
+        <v/>
+      </c>
+      <c r="M106">
+        <v>4</v>
+      </c>
+      <c r="N106" t="str">
+        <v/>
+      </c>
+      <c r="O106" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P106">
+        <v>1</v>
+      </c>
+      <c r="Q106" t="str">
+        <v/>
+      </c>
+      <c r="R106">
+        <v>1</v>
+      </c>
+      <c r="S106" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T106" t="str">
+        <v/>
+      </c>
+      <c r="U106">
+        <v>9999</v>
+      </c>
+      <c r="V106">
+        <v>1</v>
+      </c>
+      <c r="W106">
+        <v>0.5</v>
+      </c>
+      <c r="X106" t="str">
+        <v/>
+      </c>
+      <c r="Y106" t="str">
+        <v/>
+      </c>
+      <c r="Z106">
+        <v>-1</v>
+      </c>
+      <c r="AA106" t="str">
+        <v>dropbar/icon_type_1</v>
+      </c>
+      <c r="AB106" t="str">
+        <v/>
+      </c>
+      <c r="AC106" t="str">
+        <v/>
+      </c>
+      <c r="AD106">
+        <v>0</v>
+      </c>
+      <c r="AE106" t="str">
+        <v/>
+      </c>
+      <c r="AF106" t="str">
+        <v/>
+      </c>
+      <c r="AG106" t="str">
+        <v/>
+      </c>
+      <c r="AH106" t="str">
+        <v/>
+      </c>
+      <c r="AI106" t="str">
+        <v/>
+      </c>
+      <c r="AJ106">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107">
+        <v>1100205</v>
+      </c>
+      <c r="B107" t="str">
+        <v>混沌长剑</v>
+      </c>
+      <c r="C107" t="str">
+        <v/>
+      </c>
+      <c r="D107" t="str">
+        <v/>
+      </c>
+      <c r="E107" t="str">
+        <v>1</v>
+      </c>
+      <c r="F107" t="str">
+        <v>混沌长剑</v>
+      </c>
+      <c r="G107" t="str">
+        <v>zhuangbei/107/106</v>
+      </c>
+      <c r="H107" t="str">
+        <v>zhuangbei/107/106_big</v>
+      </c>
+      <c r="I107" t="str">
+        <v/>
+      </c>
+      <c r="J107" t="str">
+        <v/>
+      </c>
+      <c r="K107" t="str">
+        <v/>
+      </c>
+      <c r="L107" t="str">
+        <v/>
+      </c>
+      <c r="M107">
+        <v>4</v>
+      </c>
+      <c r="N107" t="str">
+        <v/>
+      </c>
+      <c r="O107" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P107">
+        <v>1</v>
+      </c>
+      <c r="Q107" t="str">
+        <v/>
+      </c>
+      <c r="R107">
+        <v>1</v>
+      </c>
+      <c r="S107" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T107" t="str">
+        <v/>
+      </c>
+      <c r="U107">
+        <v>9999</v>
+      </c>
+      <c r="V107">
+        <v>1</v>
+      </c>
+      <c r="W107">
+        <v>0.5</v>
+      </c>
+      <c r="X107" t="str">
+        <v/>
+      </c>
+      <c r="Y107" t="str">
+        <v/>
+      </c>
+      <c r="Z107">
+        <v>-1</v>
+      </c>
+      <c r="AA107" t="str">
+        <v>dropbar/icon_type_1</v>
+      </c>
+      <c r="AB107" t="str">
+        <v/>
+      </c>
+      <c r="AC107" t="str">
+        <v/>
+      </c>
+      <c r="AD107">
+        <v>0</v>
+      </c>
+      <c r="AE107" t="str">
+        <v/>
+      </c>
+      <c r="AF107" t="str">
+        <v/>
+      </c>
+      <c r="AG107" t="str">
+        <v/>
+      </c>
+      <c r="AH107" t="str">
+        <v/>
+      </c>
+      <c r="AI107" t="str">
+        <v/>
+      </c>
+      <c r="AJ107">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108">
+        <v>1100301</v>
+      </c>
+      <c r="B108" t="str">
+        <v>物理魔典</v>
+      </c>
+      <c r="C108" t="str">
+        <v/>
+      </c>
+      <c r="D108" t="str">
+        <v/>
+      </c>
+      <c r="E108" t="str">
+        <v>1</v>
+      </c>
+      <c r="F108" t="str">
+        <v>物理魔典</v>
+      </c>
+      <c r="G108" t="str">
+        <v>zhuangbei/101/112</v>
+      </c>
+      <c r="H108" t="str">
+        <v>zhuangbei/101/112_big</v>
+      </c>
+      <c r="I108" t="str">
+        <v/>
+      </c>
+      <c r="J108" t="str">
+        <v/>
+      </c>
+      <c r="K108" t="str">
+        <v/>
+      </c>
+      <c r="L108" t="str">
+        <v/>
+      </c>
+      <c r="M108">
+        <v>4</v>
+      </c>
+      <c r="N108" t="str">
+        <v/>
+      </c>
+      <c r="O108" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P108">
+        <v>1</v>
+      </c>
+      <c r="Q108" t="str">
+        <v/>
+      </c>
+      <c r="R108">
+        <v>1</v>
+      </c>
+      <c r="S108" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T108" t="str">
+        <v/>
+      </c>
+      <c r="U108">
+        <v>9999</v>
+      </c>
+      <c r="V108">
+        <v>1</v>
+      </c>
+      <c r="W108">
+        <v>0.5</v>
+      </c>
+      <c r="X108" t="str">
+        <v/>
+      </c>
+      <c r="Y108" t="str">
+        <v/>
+      </c>
+      <c r="Z108">
+        <v>-1</v>
+      </c>
+      <c r="AA108" t="str">
+        <v>dropbar/icon_type_1</v>
+      </c>
+      <c r="AB108" t="str">
+        <v/>
+      </c>
+      <c r="AC108" t="str">
+        <v/>
+      </c>
+      <c r="AD108">
+        <v>0</v>
+      </c>
+      <c r="AE108" t="str">
+        <v/>
+      </c>
+      <c r="AF108" t="str">
+        <v/>
+      </c>
+      <c r="AG108" t="str">
+        <v/>
+      </c>
+      <c r="AH108" t="str">
+        <v/>
+      </c>
+      <c r="AI108" t="str">
+        <v/>
+      </c>
+      <c r="AJ108">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109">
+        <v>1100302</v>
+      </c>
+      <c r="B109" t="str">
+        <v>火焰魔典</v>
+      </c>
+      <c r="C109" t="str">
+        <v/>
+      </c>
+      <c r="D109" t="str">
+        <v/>
+      </c>
+      <c r="E109" t="str">
+        <v>1</v>
+      </c>
+      <c r="F109" t="str">
+        <v>火焰魔典</v>
+      </c>
+      <c r="G109" t="str">
+        <v>zhuangbei/108/112</v>
+      </c>
+      <c r="H109" t="str">
+        <v>zhuangbei/108/112_big</v>
+      </c>
+      <c r="I109" t="str">
+        <v/>
+      </c>
+      <c r="J109" t="str">
+        <v/>
+      </c>
+      <c r="K109" t="str">
+        <v/>
+      </c>
+      <c r="L109" t="str">
+        <v/>
+      </c>
+      <c r="M109">
+        <v>4</v>
+      </c>
+      <c r="N109" t="str">
+        <v/>
+      </c>
+      <c r="O109" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P109">
+        <v>1</v>
+      </c>
+      <c r="Q109" t="str">
+        <v/>
+      </c>
+      <c r="R109">
+        <v>1</v>
+      </c>
+      <c r="S109" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T109" t="str">
+        <v/>
+      </c>
+      <c r="U109">
+        <v>9999</v>
+      </c>
+      <c r="V109">
+        <v>1</v>
+      </c>
+      <c r="W109">
+        <v>0.5</v>
+      </c>
+      <c r="X109" t="str">
+        <v/>
+      </c>
+      <c r="Y109" t="str">
+        <v/>
+      </c>
+      <c r="Z109">
+        <v>-1</v>
+      </c>
+      <c r="AA109" t="str">
+        <v>dropbar/icon_type_1</v>
+      </c>
+      <c r="AB109" t="str">
+        <v/>
+      </c>
+      <c r="AC109" t="str">
+        <v/>
+      </c>
+      <c r="AD109">
+        <v>0</v>
+      </c>
+      <c r="AE109" t="str">
+        <v/>
+      </c>
+      <c r="AF109" t="str">
+        <v/>
+      </c>
+      <c r="AG109" t="str">
+        <v/>
+      </c>
+      <c r="AH109" t="str">
+        <v/>
+      </c>
+      <c r="AI109" t="str">
+        <v/>
+      </c>
+      <c r="AJ109">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110">
+        <v>1100303</v>
+      </c>
+      <c r="B110" t="str">
+        <v>冰霜魔典</v>
+      </c>
+      <c r="C110" t="str">
+        <v/>
+      </c>
+      <c r="D110" t="str">
+        <v/>
+      </c>
+      <c r="E110" t="str">
+        <v>1</v>
+      </c>
+      <c r="F110" t="str">
+        <v>冰霜魔典</v>
+      </c>
+      <c r="G110" t="str">
+        <v>zhuangbei/106/112</v>
+      </c>
+      <c r="H110" t="str">
+        <v>zhuangbei/106/112_big</v>
+      </c>
+      <c r="I110" t="str">
+        <v/>
+      </c>
+      <c r="J110" t="str">
+        <v/>
+      </c>
+      <c r="K110" t="str">
+        <v/>
+      </c>
+      <c r="L110" t="str">
+        <v/>
+      </c>
+      <c r="M110">
+        <v>4</v>
+      </c>
+      <c r="N110" t="str">
+        <v/>
+      </c>
+      <c r="O110" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P110">
+        <v>1</v>
+      </c>
+      <c r="Q110" t="str">
+        <v/>
+      </c>
+      <c r="R110">
+        <v>1</v>
+      </c>
+      <c r="S110" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T110" t="str">
+        <v/>
+      </c>
+      <c r="U110">
+        <v>9999</v>
+      </c>
+      <c r="V110">
+        <v>1</v>
+      </c>
+      <c r="W110">
+        <v>0.5</v>
+      </c>
+      <c r="X110" t="str">
+        <v/>
+      </c>
+      <c r="Y110" t="str">
+        <v/>
+      </c>
+      <c r="Z110">
+        <v>-1</v>
+      </c>
+      <c r="AA110" t="str">
+        <v>dropbar/icon_type_1</v>
+      </c>
+      <c r="AB110" t="str">
+        <v/>
+      </c>
+      <c r="AC110" t="str">
+        <v/>
+      </c>
+      <c r="AD110">
+        <v>0</v>
+      </c>
+      <c r="AE110" t="str">
+        <v/>
+      </c>
+      <c r="AF110" t="str">
+        <v/>
+      </c>
+      <c r="AG110" t="str">
+        <v/>
+      </c>
+      <c r="AH110" t="str">
+        <v/>
+      </c>
+      <c r="AI110" t="str">
+        <v/>
+      </c>
+      <c r="AJ110">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111">
+        <v>1100304</v>
+      </c>
+      <c r="B111" t="str">
+        <v>闪电魔典</v>
+      </c>
+      <c r="C111" t="str">
+        <v/>
+      </c>
+      <c r="D111" t="str">
+        <v/>
+      </c>
+      <c r="E111" t="str">
+        <v>1</v>
+      </c>
+      <c r="F111" t="str">
+        <v>闪电魔典</v>
+      </c>
+      <c r="G111" t="str">
+        <v>zhuangbei/110/112</v>
+      </c>
+      <c r="H111" t="str">
+        <v>zhuangbei/110/112_big</v>
+      </c>
+      <c r="I111" t="str">
+        <v/>
+      </c>
+      <c r="J111" t="str">
+        <v/>
+      </c>
+      <c r="K111" t="str">
+        <v/>
+      </c>
+      <c r="L111" t="str">
+        <v/>
+      </c>
+      <c r="M111">
+        <v>4</v>
+      </c>
+      <c r="N111" t="str">
+        <v/>
+      </c>
+      <c r="O111" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P111">
+        <v>1</v>
+      </c>
+      <c r="Q111" t="str">
+        <v/>
+      </c>
+      <c r="R111">
+        <v>1</v>
+      </c>
+      <c r="S111" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T111" t="str">
+        <v/>
+      </c>
+      <c r="U111">
+        <v>9999</v>
+      </c>
+      <c r="V111">
+        <v>1</v>
+      </c>
+      <c r="W111">
+        <v>0.5</v>
+      </c>
+      <c r="X111" t="str">
+        <v/>
+      </c>
+      <c r="Y111" t="str">
+        <v/>
+      </c>
+      <c r="Z111">
+        <v>-1</v>
+      </c>
+      <c r="AA111" t="str">
+        <v>dropbar/icon_type_1</v>
+      </c>
+      <c r="AB111" t="str">
+        <v/>
+      </c>
+      <c r="AC111" t="str">
+        <v/>
+      </c>
+      <c r="AD111">
+        <v>0</v>
+      </c>
+      <c r="AE111" t="str">
+        <v/>
+      </c>
+      <c r="AF111" t="str">
+        <v/>
+      </c>
+      <c r="AG111" t="str">
+        <v/>
+      </c>
+      <c r="AH111" t="str">
+        <v/>
+      </c>
+      <c r="AI111" t="str">
+        <v/>
+      </c>
+      <c r="AJ111">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112">
+        <v>1100305</v>
+      </c>
+      <c r="B112" t="str">
+        <v>混沌魔典</v>
+      </c>
+      <c r="C112" t="str">
+        <v/>
+      </c>
+      <c r="D112" t="str">
+        <v/>
+      </c>
+      <c r="E112" t="str">
+        <v>1</v>
+      </c>
+      <c r="F112" t="str">
+        <v>混沌魔典</v>
+      </c>
+      <c r="G112" t="str">
+        <v>zhuangbei/107/112</v>
+      </c>
+      <c r="H112" t="str">
+        <v>zhuangbei/107/112_big</v>
+      </c>
+      <c r="I112" t="str">
+        <v/>
+      </c>
+      <c r="J112" t="str">
+        <v/>
+      </c>
+      <c r="K112" t="str">
+        <v/>
+      </c>
+      <c r="L112" t="str">
+        <v/>
+      </c>
+      <c r="M112">
+        <v>4</v>
+      </c>
+      <c r="N112" t="str">
+        <v/>
+      </c>
+      <c r="O112" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P112">
+        <v>1</v>
+      </c>
+      <c r="Q112" t="str">
+        <v/>
+      </c>
+      <c r="R112">
+        <v>1</v>
+      </c>
+      <c r="S112" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T112" t="str">
+        <v/>
+      </c>
+      <c r="U112">
+        <v>9999</v>
+      </c>
+      <c r="V112">
+        <v>1</v>
+      </c>
+      <c r="W112">
+        <v>0.5</v>
+      </c>
+      <c r="X112" t="str">
+        <v/>
+      </c>
+      <c r="Y112" t="str">
+        <v/>
+      </c>
+      <c r="Z112">
+        <v>-1</v>
+      </c>
+      <c r="AA112" t="str">
+        <v>dropbar/icon_type_1</v>
+      </c>
+      <c r="AB112" t="str">
+        <v/>
+      </c>
+      <c r="AC112" t="str">
+        <v/>
+      </c>
+      <c r="AD112">
+        <v>0</v>
+      </c>
+      <c r="AE112" t="str">
+        <v/>
+      </c>
+      <c r="AF112" t="str">
+        <v/>
+      </c>
+      <c r="AG112" t="str">
+        <v/>
+      </c>
+      <c r="AH112" t="str">
+        <v/>
+      </c>
+      <c r="AI112" t="str">
+        <v/>
+      </c>
+      <c r="AJ112">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113">
+        <v>1200101</v>
+      </c>
+      <c r="B113" t="str">
+        <v>铸铁头盔</v>
+      </c>
+      <c r="C113" t="str">
+        <v/>
+      </c>
+      <c r="D113" t="str">
+        <v/>
+      </c>
+      <c r="E113" t="str">
+        <v>1</v>
+      </c>
+      <c r="F113" t="str">
+        <v>铸铁头盔</v>
+      </c>
+      <c r="G113" t="str">
+        <v>zhuangbei/101/201</v>
+      </c>
+      <c r="H113" t="str">
+        <v/>
+      </c>
+      <c r="I113" t="str">
+        <v/>
+      </c>
+      <c r="J113" t="str">
+        <v/>
+      </c>
+      <c r="K113" t="str">
+        <v/>
+      </c>
+      <c r="L113" t="str">
+        <v/>
+      </c>
+      <c r="M113">
+        <v>4</v>
+      </c>
+      <c r="N113" t="str">
+        <v/>
+      </c>
+      <c r="O113" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P113">
+        <v>1</v>
+      </c>
+      <c r="Q113" t="str">
+        <v/>
+      </c>
+      <c r="R113">
+        <v>1</v>
+      </c>
+      <c r="S113" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T113" t="str">
+        <v/>
+      </c>
+      <c r="U113">
+        <v>9999</v>
+      </c>
+      <c r="V113">
+        <v>1</v>
+      </c>
+      <c r="W113">
+        <v>0.5</v>
+      </c>
+      <c r="X113" t="str">
+        <v/>
+      </c>
+      <c r="Y113" t="str">
+        <v/>
+      </c>
+      <c r="Z113">
+        <v>-1</v>
+      </c>
+      <c r="AA113" t="str">
+        <v>dropbar/icon_type_2</v>
+      </c>
+      <c r="AB113" t="str">
+        <v/>
+      </c>
+      <c r="AC113" t="str">
+        <v/>
+      </c>
+      <c r="AD113">
+        <v>0</v>
+      </c>
+      <c r="AE113" t="str">
+        <v/>
+      </c>
+      <c r="AF113" t="str">
+        <v/>
+      </c>
+      <c r="AG113" t="str">
+        <v/>
+      </c>
+      <c r="AH113" t="str">
+        <v/>
+      </c>
+      <c r="AI113" t="str">
+        <v/>
+      </c>
+      <c r="AJ113">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114">
+        <v>1200102</v>
+      </c>
+      <c r="B114" t="str">
+        <v>银制头盔</v>
+      </c>
+      <c r="C114" t="str">
+        <v/>
+      </c>
+      <c r="D114" t="str">
+        <v/>
+      </c>
+      <c r="E114" t="str">
+        <v>1</v>
+      </c>
+      <c r="F114" t="str">
+        <v>银制头盔</v>
+      </c>
+      <c r="G114" t="str">
+        <v>zhuangbei/101/201</v>
+      </c>
+      <c r="H114" t="str">
+        <v/>
+      </c>
+      <c r="I114" t="str">
+        <v/>
+      </c>
+      <c r="J114" t="str">
+        <v/>
+      </c>
+      <c r="K114" t="str">
+        <v/>
+      </c>
+      <c r="L114" t="str">
+        <v/>
+      </c>
+      <c r="M114">
+        <v>4</v>
+      </c>
+      <c r="N114" t="str">
+        <v/>
+      </c>
+      <c r="O114" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P114">
+        <v>1</v>
+      </c>
+      <c r="Q114" t="str">
+        <v/>
+      </c>
+      <c r="R114">
+        <v>1</v>
+      </c>
+      <c r="S114" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T114" t="str">
+        <v/>
+      </c>
+      <c r="U114">
+        <v>9999</v>
+      </c>
+      <c r="V114">
+        <v>1</v>
+      </c>
+      <c r="W114">
+        <v>0.5</v>
+      </c>
+      <c r="X114" t="str">
+        <v/>
+      </c>
+      <c r="Y114" t="str">
+        <v/>
+      </c>
+      <c r="Z114">
+        <v>-1</v>
+      </c>
+      <c r="AA114" t="str">
+        <v>dropbar/icon_type_2</v>
+      </c>
+      <c r="AB114" t="str">
+        <v/>
+      </c>
+      <c r="AC114" t="str">
+        <v/>
+      </c>
+      <c r="AD114">
+        <v>0</v>
+      </c>
+      <c r="AE114" t="str">
+        <v/>
+      </c>
+      <c r="AF114" t="str">
+        <v/>
+      </c>
+      <c r="AG114" t="str">
+        <v/>
+      </c>
+      <c r="AH114" t="str">
+        <v/>
+      </c>
+      <c r="AI114" t="str">
+        <v/>
+      </c>
+      <c r="AJ114">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115">
+        <v>1300101</v>
+      </c>
+      <c r="B115" t="str">
+        <v>铸铁胸甲</v>
+      </c>
+      <c r="C115" t="str">
+        <v/>
+      </c>
+      <c r="D115" t="str">
+        <v/>
+      </c>
+      <c r="E115" t="str">
+        <v>1</v>
+      </c>
+      <c r="F115" t="str">
+        <v>铸铁胸甲</v>
+      </c>
+      <c r="G115" t="str">
+        <v>zhuangbei/101/301</v>
+      </c>
+      <c r="H115" t="str">
+        <v/>
+      </c>
+      <c r="I115" t="str">
+        <v/>
+      </c>
+      <c r="J115" t="str">
+        <v/>
+      </c>
+      <c r="K115" t="str">
+        <v/>
+      </c>
+      <c r="L115" t="str">
+        <v/>
+      </c>
+      <c r="M115">
+        <v>4</v>
+      </c>
+      <c r="N115" t="str">
+        <v/>
+      </c>
+      <c r="O115" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P115">
+        <v>1</v>
+      </c>
+      <c r="Q115" t="str">
+        <v/>
+      </c>
+      <c r="R115">
+        <v>1</v>
+      </c>
+      <c r="S115" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T115" t="str">
+        <v/>
+      </c>
+      <c r="U115">
+        <v>9999</v>
+      </c>
+      <c r="V115">
+        <v>1</v>
+      </c>
+      <c r="W115">
+        <v>0.5</v>
+      </c>
+      <c r="X115" t="str">
+        <v/>
+      </c>
+      <c r="Y115" t="str">
+        <v/>
+      </c>
+      <c r="Z115">
+        <v>-1</v>
+      </c>
+      <c r="AA115" t="str">
+        <v>dropbar/icon_type_3</v>
+      </c>
+      <c r="AB115" t="str">
+        <v/>
+      </c>
+      <c r="AC115" t="str">
+        <v/>
+      </c>
+      <c r="AD115">
+        <v>0</v>
+      </c>
+      <c r="AE115" t="str">
+        <v/>
+      </c>
+      <c r="AF115" t="str">
+        <v/>
+      </c>
+      <c r="AG115" t="str">
+        <v/>
+      </c>
+      <c r="AH115" t="str">
+        <v/>
+      </c>
+      <c r="AI115" t="str">
+        <v/>
+      </c>
+      <c r="AJ115">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116">
+        <v>1300102</v>
+      </c>
+      <c r="B116" t="str">
+        <v>皮制胸甲</v>
+      </c>
+      <c r="C116" t="str">
+        <v/>
+      </c>
+      <c r="D116" t="str">
+        <v/>
+      </c>
+      <c r="E116" t="str">
+        <v>1</v>
+      </c>
+      <c r="F116" t="str">
+        <v>皮制胸甲</v>
+      </c>
+      <c r="G116" t="str">
+        <v>zhuangbei/101/301</v>
+      </c>
+      <c r="H116" t="str">
+        <v/>
+      </c>
+      <c r="I116" t="str">
+        <v/>
+      </c>
+      <c r="J116" t="str">
+        <v/>
+      </c>
+      <c r="K116" t="str">
+        <v/>
+      </c>
+      <c r="L116" t="str">
+        <v/>
+      </c>
+      <c r="M116">
+        <v>4</v>
+      </c>
+      <c r="N116" t="str">
+        <v/>
+      </c>
+      <c r="O116" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P116">
+        <v>1</v>
+      </c>
+      <c r="Q116" t="str">
+        <v/>
+      </c>
+      <c r="R116">
+        <v>1</v>
+      </c>
+      <c r="S116" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T116" t="str">
+        <v/>
+      </c>
+      <c r="U116">
+        <v>9999</v>
+      </c>
+      <c r="V116">
+        <v>1</v>
+      </c>
+      <c r="W116">
+        <v>0.5</v>
+      </c>
+      <c r="X116" t="str">
+        <v/>
+      </c>
+      <c r="Y116" t="str">
+        <v/>
+      </c>
+      <c r="Z116">
+        <v>-1</v>
+      </c>
+      <c r="AA116" t="str">
+        <v>dropbar/icon_type_3</v>
+      </c>
+      <c r="AB116" t="str">
+        <v/>
+      </c>
+      <c r="AC116" t="str">
+        <v/>
+      </c>
+      <c r="AD116">
+        <v>0</v>
+      </c>
+      <c r="AE116" t="str">
+        <v/>
+      </c>
+      <c r="AF116" t="str">
+        <v/>
+      </c>
+      <c r="AG116" t="str">
+        <v/>
+      </c>
+      <c r="AH116" t="str">
+        <v/>
+      </c>
+      <c r="AI116" t="str">
+        <v/>
+      </c>
+      <c r="AJ116">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117">
+        <v>1300103</v>
+      </c>
+      <c r="B117" t="str">
+        <v>铁锁胸甲</v>
+      </c>
+      <c r="C117" t="str">
+        <v/>
+      </c>
+      <c r="D117" t="str">
+        <v/>
+      </c>
+      <c r="E117" t="str">
+        <v>1</v>
+      </c>
+      <c r="F117" t="str">
+        <v>铁锁胸甲</v>
+      </c>
+      <c r="G117" t="str">
+        <v>zhuangbei/101/301</v>
+      </c>
+      <c r="H117" t="str">
+        <v/>
+      </c>
+      <c r="I117" t="str">
+        <v/>
+      </c>
+      <c r="J117" t="str">
+        <v/>
+      </c>
+      <c r="K117" t="str">
+        <v/>
+      </c>
+      <c r="L117" t="str">
+        <v/>
+      </c>
+      <c r="M117">
+        <v>4</v>
+      </c>
+      <c r="N117" t="str">
+        <v/>
+      </c>
+      <c r="O117" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P117">
+        <v>1</v>
+      </c>
+      <c r="Q117" t="str">
+        <v/>
+      </c>
+      <c r="R117">
+        <v>1</v>
+      </c>
+      <c r="S117" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T117" t="str">
+        <v/>
+      </c>
+      <c r="U117">
+        <v>9999</v>
+      </c>
+      <c r="V117">
+        <v>1</v>
+      </c>
+      <c r="W117">
+        <v>0.5</v>
+      </c>
+      <c r="X117" t="str">
+        <v/>
+      </c>
+      <c r="Y117" t="str">
+        <v/>
+      </c>
+      <c r="Z117">
+        <v>-1</v>
+      </c>
+      <c r="AA117" t="str">
+        <v>dropbar/icon_type_3</v>
+      </c>
+      <c r="AB117" t="str">
+        <v/>
+      </c>
+      <c r="AC117" t="str">
+        <v/>
+      </c>
+      <c r="AD117">
+        <v>0</v>
+      </c>
+      <c r="AE117" t="str">
+        <v/>
+      </c>
+      <c r="AF117" t="str">
+        <v/>
+      </c>
+      <c r="AG117" t="str">
+        <v/>
+      </c>
+      <c r="AH117" t="str">
+        <v/>
+      </c>
+      <c r="AI117" t="str">
+        <v/>
+      </c>
+      <c r="AJ117">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118">
+        <v>1400101</v>
+      </c>
+      <c r="B118" t="str">
+        <v>铸铁腿甲</v>
+      </c>
+      <c r="C118" t="str">
+        <v/>
+      </c>
+      <c r="D118" t="str">
+        <v/>
+      </c>
+      <c r="E118" t="str">
+        <v>1</v>
+      </c>
+      <c r="F118" t="str">
+        <v>铸铁腿甲</v>
+      </c>
+      <c r="G118" t="str">
+        <v>zhuangbei/101/1201</v>
+      </c>
+      <c r="H118" t="str">
+        <v/>
+      </c>
+      <c r="I118" t="str">
+        <v/>
+      </c>
+      <c r="J118" t="str">
+        <v/>
+      </c>
+      <c r="K118" t="str">
+        <v/>
+      </c>
+      <c r="L118" t="str">
+        <v/>
+      </c>
+      <c r="M118">
+        <v>4</v>
+      </c>
+      <c r="N118" t="str">
+        <v/>
+      </c>
+      <c r="O118" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P118">
+        <v>1</v>
+      </c>
+      <c r="Q118" t="str">
+        <v/>
+      </c>
+      <c r="R118">
+        <v>1</v>
+      </c>
+      <c r="S118" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T118" t="str">
+        <v/>
+      </c>
+      <c r="U118">
+        <v>9999</v>
+      </c>
+      <c r="V118">
+        <v>1</v>
+      </c>
+      <c r="W118">
+        <v>0.5</v>
+      </c>
+      <c r="X118" t="str">
+        <v/>
+      </c>
+      <c r="Y118" t="str">
+        <v/>
+      </c>
+      <c r="Z118">
+        <v>-1</v>
+      </c>
+      <c r="AA118" t="str">
+        <v>dropbar/icon_type_12</v>
+      </c>
+      <c r="AB118" t="str">
+        <v/>
+      </c>
+      <c r="AC118" t="str">
+        <v/>
+      </c>
+      <c r="AD118">
+        <v>0</v>
+      </c>
+      <c r="AE118" t="str">
+        <v/>
+      </c>
+      <c r="AF118" t="str">
+        <v/>
+      </c>
+      <c r="AG118" t="str">
+        <v/>
+      </c>
+      <c r="AH118" t="str">
+        <v/>
+      </c>
+      <c r="AI118" t="str">
+        <v/>
+      </c>
+      <c r="AJ118">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119">
+        <v>1400102</v>
+      </c>
+      <c r="B119" t="str">
+        <v>钢制腿甲</v>
+      </c>
+      <c r="C119" t="str">
+        <v/>
+      </c>
+      <c r="D119" t="str">
+        <v/>
+      </c>
+      <c r="E119" t="str">
+        <v>1</v>
+      </c>
+      <c r="F119" t="str">
+        <v>钢制腿甲</v>
+      </c>
+      <c r="G119" t="str">
+        <v>zhuangbei/101/1201</v>
+      </c>
+      <c r="H119" t="str">
+        <v/>
+      </c>
+      <c r="I119" t="str">
+        <v/>
+      </c>
+      <c r="J119" t="str">
+        <v/>
+      </c>
+      <c r="K119" t="str">
+        <v/>
+      </c>
+      <c r="L119" t="str">
+        <v/>
+      </c>
+      <c r="M119">
+        <v>4</v>
+      </c>
+      <c r="N119" t="str">
+        <v/>
+      </c>
+      <c r="O119" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P119">
+        <v>1</v>
+      </c>
+      <c r="Q119" t="str">
+        <v/>
+      </c>
+      <c r="R119">
+        <v>1</v>
+      </c>
+      <c r="S119" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T119" t="str">
+        <v/>
+      </c>
+      <c r="U119">
+        <v>9999</v>
+      </c>
+      <c r="V119">
+        <v>1</v>
+      </c>
+      <c r="W119">
+        <v>0.5</v>
+      </c>
+      <c r="X119" t="str">
+        <v/>
+      </c>
+      <c r="Y119" t="str">
+        <v/>
+      </c>
+      <c r="Z119">
+        <v>-1</v>
+      </c>
+      <c r="AA119" t="str">
+        <v>dropbar/icon_type_12</v>
+      </c>
+      <c r="AB119" t="str">
+        <v/>
+      </c>
+      <c r="AC119" t="str">
+        <v/>
+      </c>
+      <c r="AD119">
+        <v>0</v>
+      </c>
+      <c r="AE119" t="str">
+        <v/>
+      </c>
+      <c r="AF119" t="str">
+        <v/>
+      </c>
+      <c r="AG119" t="str">
+        <v/>
+      </c>
+      <c r="AH119" t="str">
+        <v/>
+      </c>
+      <c r="AI119" t="str">
+        <v/>
+      </c>
+      <c r="AJ119">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120">
+        <v>1500101</v>
+      </c>
+      <c r="B120" t="str">
+        <v>铸铁靴</v>
+      </c>
+      <c r="C120" t="str">
+        <v/>
+      </c>
+      <c r="D120" t="str">
+        <v/>
+      </c>
+      <c r="E120" t="str">
+        <v>1</v>
+      </c>
+      <c r="F120" t="str">
+        <v>铸铁靴</v>
+      </c>
+      <c r="G120" t="str">
+        <v>zhuangbei/101/401</v>
+      </c>
+      <c r="H120" t="str">
+        <v/>
+      </c>
+      <c r="I120" t="str">
+        <v/>
+      </c>
+      <c r="J120" t="str">
+        <v/>
+      </c>
+      <c r="K120" t="str">
+        <v/>
+      </c>
+      <c r="L120" t="str">
+        <v/>
+      </c>
+      <c r="M120">
+        <v>4</v>
+      </c>
+      <c r="N120" t="str">
+        <v/>
+      </c>
+      <c r="O120" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P120">
+        <v>1</v>
+      </c>
+      <c r="Q120" t="str">
+        <v/>
+      </c>
+      <c r="R120">
+        <v>1</v>
+      </c>
+      <c r="S120" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T120" t="str">
+        <v/>
+      </c>
+      <c r="U120">
+        <v>9999</v>
+      </c>
+      <c r="V120">
+        <v>1</v>
+      </c>
+      <c r="W120">
+        <v>0.5</v>
+      </c>
+      <c r="X120" t="str">
+        <v/>
+      </c>
+      <c r="Y120" t="str">
+        <v/>
+      </c>
+      <c r="Z120">
+        <v>-1</v>
+      </c>
+      <c r="AA120" t="str">
+        <v>dropbar/icon_type_4</v>
+      </c>
+      <c r="AB120" t="str">
+        <v/>
+      </c>
+      <c r="AC120" t="str">
+        <v/>
+      </c>
+      <c r="AD120">
+        <v>0</v>
+      </c>
+      <c r="AE120" t="str">
+        <v/>
+      </c>
+      <c r="AF120" t="str">
+        <v/>
+      </c>
+      <c r="AG120" t="str">
+        <v/>
+      </c>
+      <c r="AH120" t="str">
+        <v/>
+      </c>
+      <c r="AI120" t="str">
+        <v/>
+      </c>
+      <c r="AJ120">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121">
+        <v>1500102</v>
+      </c>
+      <c r="B121" t="str">
+        <v>鞣制靴</v>
+      </c>
+      <c r="C121" t="str">
+        <v/>
+      </c>
+      <c r="D121" t="str">
+        <v/>
+      </c>
+      <c r="E121" t="str">
+        <v>1</v>
+      </c>
+      <c r="F121" t="str">
+        <v>鞣制靴</v>
+      </c>
+      <c r="G121" t="str">
+        <v>zhuangbei/101/401</v>
+      </c>
+      <c r="H121" t="str">
+        <v/>
+      </c>
+      <c r="I121" t="str">
+        <v/>
+      </c>
+      <c r="J121" t="str">
+        <v/>
+      </c>
+      <c r="K121" t="str">
+        <v/>
+      </c>
+      <c r="L121" t="str">
+        <v/>
+      </c>
+      <c r="M121">
+        <v>4</v>
+      </c>
+      <c r="N121" t="str">
+        <v/>
+      </c>
+      <c r="O121" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P121">
+        <v>1</v>
+      </c>
+      <c r="Q121" t="str">
+        <v/>
+      </c>
+      <c r="R121">
+        <v>1</v>
+      </c>
+      <c r="S121" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T121" t="str">
+        <v/>
+      </c>
+      <c r="U121">
+        <v>9999</v>
+      </c>
+      <c r="V121">
+        <v>1</v>
+      </c>
+      <c r="W121">
+        <v>0.5</v>
+      </c>
+      <c r="X121" t="str">
+        <v/>
+      </c>
+      <c r="Y121" t="str">
+        <v/>
+      </c>
+      <c r="Z121">
+        <v>-1</v>
+      </c>
+      <c r="AA121" t="str">
+        <v>dropbar/icon_type_4</v>
+      </c>
+      <c r="AB121" t="str">
+        <v/>
+      </c>
+      <c r="AC121" t="str">
+        <v/>
+      </c>
+      <c r="AD121">
+        <v>0</v>
+      </c>
+      <c r="AE121" t="str">
+        <v/>
+      </c>
+      <c r="AF121" t="str">
+        <v/>
+      </c>
+      <c r="AG121" t="str">
+        <v/>
+      </c>
+      <c r="AH121" t="str">
+        <v/>
+      </c>
+      <c r="AI121" t="str">
+        <v/>
+      </c>
+      <c r="AJ121">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122">
+        <v>1500103</v>
+      </c>
+      <c r="B122" t="str">
+        <v>符文靴</v>
+      </c>
+      <c r="C122" t="str">
+        <v/>
+      </c>
+      <c r="D122" t="str">
+        <v/>
+      </c>
+      <c r="E122" t="str">
+        <v>1</v>
+      </c>
+      <c r="F122" t="str">
+        <v>符文靴</v>
+      </c>
+      <c r="G122" t="str">
+        <v>zhuangbei/101/401</v>
+      </c>
+      <c r="H122" t="str">
+        <v/>
+      </c>
+      <c r="I122" t="str">
+        <v/>
+      </c>
+      <c r="J122" t="str">
+        <v/>
+      </c>
+      <c r="K122" t="str">
+        <v/>
+      </c>
+      <c r="L122" t="str">
+        <v/>
+      </c>
+      <c r="M122">
+        <v>4</v>
+      </c>
+      <c r="N122" t="str">
+        <v/>
+      </c>
+      <c r="O122" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P122">
+        <v>1</v>
+      </c>
+      <c r="Q122" t="str">
+        <v/>
+      </c>
+      <c r="R122">
+        <v>1</v>
+      </c>
+      <c r="S122" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T122" t="str">
+        <v/>
+      </c>
+      <c r="U122">
+        <v>9999</v>
+      </c>
+      <c r="V122">
+        <v>1</v>
+      </c>
+      <c r="W122">
+        <v>0.5</v>
+      </c>
+      <c r="X122" t="str">
+        <v/>
+      </c>
+      <c r="Y122" t="str">
+        <v/>
+      </c>
+      <c r="Z122">
+        <v>-1</v>
+      </c>
+      <c r="AA122" t="str">
+        <v>dropbar/icon_type_4</v>
+      </c>
+      <c r="AB122" t="str">
+        <v/>
+      </c>
+      <c r="AC122" t="str">
+        <v/>
+      </c>
+      <c r="AD122">
+        <v>0</v>
+      </c>
+      <c r="AE122" t="str">
+        <v/>
+      </c>
+      <c r="AF122" t="str">
+        <v/>
+      </c>
+      <c r="AG122" t="str">
+        <v/>
+      </c>
+      <c r="AH122" t="str">
+        <v/>
+      </c>
+      <c r="AI122" t="str">
+        <v/>
+      </c>
+      <c r="AJ122">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123">
+        <v>1600101</v>
+      </c>
+      <c r="B123" t="str">
+        <v>铸铁护手</v>
+      </c>
+      <c r="C123" t="str">
+        <v/>
+      </c>
+      <c r="D123" t="str">
+        <v/>
+      </c>
+      <c r="E123" t="str">
+        <v>1</v>
+      </c>
+      <c r="F123" t="str">
+        <v>铸铁护手</v>
+      </c>
+      <c r="G123" t="str">
+        <v>zhuangbei/101/501</v>
+      </c>
+      <c r="H123" t="str">
+        <v/>
+      </c>
+      <c r="I123" t="str">
+        <v/>
+      </c>
+      <c r="J123" t="str">
+        <v/>
+      </c>
+      <c r="K123" t="str">
+        <v/>
+      </c>
+      <c r="L123" t="str">
+        <v/>
+      </c>
+      <c r="M123">
+        <v>4</v>
+      </c>
+      <c r="N123" t="str">
+        <v/>
+      </c>
+      <c r="O123" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P123">
+        <v>1</v>
+      </c>
+      <c r="Q123" t="str">
+        <v/>
+      </c>
+      <c r="R123">
+        <v>1</v>
+      </c>
+      <c r="S123" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T123" t="str">
+        <v/>
+      </c>
+      <c r="U123">
+        <v>9999</v>
+      </c>
+      <c r="V123">
+        <v>1</v>
+      </c>
+      <c r="W123">
+        <v>0.5</v>
+      </c>
+      <c r="X123" t="str">
+        <v/>
+      </c>
+      <c r="Y123" t="str">
+        <v/>
+      </c>
+      <c r="Z123">
+        <v>-1</v>
+      </c>
+      <c r="AA123" t="str">
+        <v>dropbar/icon_type_5</v>
+      </c>
+      <c r="AB123" t="str">
+        <v/>
+      </c>
+      <c r="AC123" t="str">
+        <v/>
+      </c>
+      <c r="AD123">
+        <v>0</v>
+      </c>
+      <c r="AE123" t="str">
+        <v/>
+      </c>
+      <c r="AF123" t="str">
+        <v/>
+      </c>
+      <c r="AG123" t="str">
+        <v/>
+      </c>
+      <c r="AH123" t="str">
+        <v/>
+      </c>
+      <c r="AI123" t="str">
+        <v/>
+      </c>
+      <c r="AJ123">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124">
+        <v>1600102</v>
+      </c>
+      <c r="B124" t="str">
+        <v>皮制护手</v>
+      </c>
+      <c r="C124" t="str">
+        <v/>
+      </c>
+      <c r="D124" t="str">
+        <v/>
+      </c>
+      <c r="E124" t="str">
+        <v>1</v>
+      </c>
+      <c r="F124" t="str">
+        <v>皮制护手</v>
+      </c>
+      <c r="G124" t="str">
+        <v>zhuangbei/101/502</v>
+      </c>
+      <c r="H124" t="str">
+        <v/>
+      </c>
+      <c r="I124" t="str">
+        <v/>
+      </c>
+      <c r="J124" t="str">
+        <v/>
+      </c>
+      <c r="K124" t="str">
+        <v/>
+      </c>
+      <c r="L124" t="str">
+        <v/>
+      </c>
+      <c r="M124">
+        <v>4</v>
+      </c>
+      <c r="N124" t="str">
+        <v/>
+      </c>
+      <c r="O124" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P124">
+        <v>1</v>
+      </c>
+      <c r="Q124" t="str">
+        <v/>
+      </c>
+      <c r="R124">
+        <v>1</v>
+      </c>
+      <c r="S124" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T124" t="str">
+        <v/>
+      </c>
+      <c r="U124">
+        <v>9999</v>
+      </c>
+      <c r="V124">
+        <v>1</v>
+      </c>
+      <c r="W124">
+        <v>0.5</v>
+      </c>
+      <c r="X124" t="str">
+        <v/>
+      </c>
+      <c r="Y124" t="str">
+        <v/>
+      </c>
+      <c r="Z124">
+        <v>-1</v>
+      </c>
+      <c r="AA124" t="str">
+        <v>dropbar/icon_type_5</v>
+      </c>
+      <c r="AB124" t="str">
+        <v/>
+      </c>
+      <c r="AC124" t="str">
+        <v/>
+      </c>
+      <c r="AD124">
+        <v>0</v>
+      </c>
+      <c r="AE124" t="str">
+        <v/>
+      </c>
+      <c r="AF124" t="str">
+        <v/>
+      </c>
+      <c r="AG124" t="str">
+        <v/>
+      </c>
+      <c r="AH124" t="str">
+        <v/>
+      </c>
+      <c r="AI124" t="str">
+        <v/>
+      </c>
+      <c r="AJ124">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125">
+        <v>1600103</v>
+      </c>
+      <c r="B125" t="str">
+        <v>轻质护手</v>
+      </c>
+      <c r="C125" t="str">
+        <v/>
+      </c>
+      <c r="D125" t="str">
+        <v/>
+      </c>
+      <c r="E125" t="str">
+        <v>1</v>
+      </c>
+      <c r="F125" t="str">
+        <v>轻质护手</v>
+      </c>
+      <c r="G125" t="str">
+        <v>zhuangbei/101/503</v>
+      </c>
+      <c r="H125" t="str">
+        <v/>
+      </c>
+      <c r="I125" t="str">
+        <v/>
+      </c>
+      <c r="J125" t="str">
+        <v/>
+      </c>
+      <c r="K125" t="str">
+        <v/>
+      </c>
+      <c r="L125" t="str">
+        <v/>
+      </c>
+      <c r="M125">
+        <v>4</v>
+      </c>
+      <c r="N125" t="str">
+        <v/>
+      </c>
+      <c r="O125" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P125">
+        <v>1</v>
+      </c>
+      <c r="Q125" t="str">
+        <v/>
+      </c>
+      <c r="R125">
+        <v>1</v>
+      </c>
+      <c r="S125" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T125" t="str">
+        <v/>
+      </c>
+      <c r="U125">
+        <v>9999</v>
+      </c>
+      <c r="V125">
+        <v>1</v>
+      </c>
+      <c r="W125">
+        <v>0.5</v>
+      </c>
+      <c r="X125" t="str">
+        <v/>
+      </c>
+      <c r="Y125" t="str">
+        <v/>
+      </c>
+      <c r="Z125">
+        <v>-1</v>
+      </c>
+      <c r="AA125" t="str">
+        <v>dropbar/icon_type_5</v>
+      </c>
+      <c r="AB125" t="str">
+        <v/>
+      </c>
+      <c r="AC125" t="str">
+        <v/>
+      </c>
+      <c r="AD125">
+        <v>0</v>
+      </c>
+      <c r="AE125" t="str">
+        <v/>
+      </c>
+      <c r="AF125" t="str">
+        <v/>
+      </c>
+      <c r="AG125" t="str">
+        <v/>
+      </c>
+      <c r="AH125" t="str">
+        <v/>
+      </c>
+      <c r="AI125" t="str">
+        <v/>
+      </c>
+      <c r="AJ125">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126">
+        <v>1700101</v>
+      </c>
+      <c r="B126" t="str">
+        <v>精铁礼花</v>
+      </c>
+      <c r="C126" t="str">
+        <v/>
+      </c>
+      <c r="D126" t="str">
+        <v/>
+      </c>
+      <c r="E126" t="str">
+        <v>1</v>
+      </c>
+      <c r="F126" t="str">
+        <v>精铁礼花</v>
+      </c>
+      <c r="G126" t="str">
+        <v>zhuangbei/101/601</v>
+      </c>
+      <c r="H126" t="str">
+        <v/>
+      </c>
+      <c r="I126" t="str">
+        <v/>
+      </c>
+      <c r="J126" t="str">
+        <v/>
+      </c>
+      <c r="K126" t="str">
+        <v/>
+      </c>
+      <c r="L126" t="str">
+        <v/>
+      </c>
+      <c r="M126">
+        <v>4</v>
+      </c>
+      <c r="N126" t="str">
+        <v/>
+      </c>
+      <c r="O126" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P126">
+        <v>1</v>
+      </c>
+      <c r="Q126" t="str">
+        <v/>
+      </c>
+      <c r="R126">
+        <v>1</v>
+      </c>
+      <c r="S126" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T126" t="str">
+        <v/>
+      </c>
+      <c r="U126">
+        <v>9999</v>
+      </c>
+      <c r="V126">
+        <v>1</v>
+      </c>
+      <c r="W126">
+        <v>0.5</v>
+      </c>
+      <c r="X126" t="str">
+        <v/>
+      </c>
+      <c r="Y126" t="str">
+        <v/>
+      </c>
+      <c r="Z126">
+        <v>-1</v>
+      </c>
+      <c r="AA126" t="str">
+        <v>dropbar/icon_type_6</v>
+      </c>
+      <c r="AB126" t="str">
+        <v/>
+      </c>
+      <c r="AC126" t="str">
+        <v/>
+      </c>
+      <c r="AD126">
+        <v>0</v>
+      </c>
+      <c r="AE126" t="str">
+        <v/>
+      </c>
+      <c r="AF126" t="str">
+        <v/>
+      </c>
+      <c r="AG126" t="str">
+        <v/>
+      </c>
+      <c r="AH126" t="str">
+        <v/>
+      </c>
+      <c r="AI126" t="str">
+        <v/>
+      </c>
+      <c r="AJ126">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127">
+        <v>1700102</v>
+      </c>
+      <c r="B127" t="str">
+        <v>宝石礼花</v>
+      </c>
+      <c r="C127" t="str">
+        <v/>
+      </c>
+      <c r="D127" t="str">
+        <v/>
+      </c>
+      <c r="E127" t="str">
+        <v>1</v>
+      </c>
+      <c r="F127" t="str">
+        <v>宝石礼花</v>
+      </c>
+      <c r="G127" t="str">
+        <v>zhuangbei/103/601</v>
+      </c>
+      <c r="H127" t="str">
+        <v/>
+      </c>
+      <c r="I127" t="str">
+        <v/>
+      </c>
+      <c r="J127" t="str">
+        <v/>
+      </c>
+      <c r="K127" t="str">
+        <v/>
+      </c>
+      <c r="L127" t="str">
+        <v/>
+      </c>
+      <c r="M127">
+        <v>4</v>
+      </c>
+      <c r="N127" t="str">
+        <v/>
+      </c>
+      <c r="O127" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P127">
+        <v>1</v>
+      </c>
+      <c r="Q127" t="str">
+        <v/>
+      </c>
+      <c r="R127">
+        <v>1</v>
+      </c>
+      <c r="S127" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T127" t="str">
+        <v/>
+      </c>
+      <c r="U127">
+        <v>9999</v>
+      </c>
+      <c r="V127">
+        <v>1</v>
+      </c>
+      <c r="W127">
+        <v>0.5</v>
+      </c>
+      <c r="X127" t="str">
+        <v/>
+      </c>
+      <c r="Y127" t="str">
+        <v/>
+      </c>
+      <c r="Z127">
+        <v>-1</v>
+      </c>
+      <c r="AA127" t="str">
+        <v>dropbar/icon_type_6</v>
+      </c>
+      <c r="AB127" t="str">
+        <v/>
+      </c>
+      <c r="AC127" t="str">
+        <v/>
+      </c>
+      <c r="AD127">
+        <v>0</v>
+      </c>
+      <c r="AE127" t="str">
+        <v/>
+      </c>
+      <c r="AF127" t="str">
+        <v/>
+      </c>
+      <c r="AG127" t="str">
+        <v/>
+      </c>
+      <c r="AH127" t="str">
+        <v/>
+      </c>
+      <c r="AI127" t="str">
+        <v/>
+      </c>
+      <c r="AJ127">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128">
+        <v>1700103</v>
+      </c>
+      <c r="B128" t="str">
+        <v>鹅绒礼花</v>
+      </c>
+      <c r="C128" t="str">
+        <v/>
+      </c>
+      <c r="D128" t="str">
+        <v/>
+      </c>
+      <c r="E128" t="str">
+        <v>1</v>
+      </c>
+      <c r="F128" t="str">
+        <v>鹅绒礼花</v>
+      </c>
+      <c r="G128" t="str">
+        <v>zhuangbei/103/601</v>
+      </c>
+      <c r="H128" t="str">
+        <v/>
+      </c>
+      <c r="I128" t="str">
+        <v/>
+      </c>
+      <c r="J128" t="str">
+        <v/>
+      </c>
+      <c r="K128" t="str">
+        <v/>
+      </c>
+      <c r="L128" t="str">
+        <v/>
+      </c>
+      <c r="M128">
+        <v>4</v>
+      </c>
+      <c r="N128" t="str">
+        <v/>
+      </c>
+      <c r="O128" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P128">
+        <v>1</v>
+      </c>
+      <c r="Q128" t="str">
+        <v/>
+      </c>
+      <c r="R128">
+        <v>1</v>
+      </c>
+      <c r="S128" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T128" t="str">
+        <v/>
+      </c>
+      <c r="U128">
+        <v>9999</v>
+      </c>
+      <c r="V128">
+        <v>1</v>
+      </c>
+      <c r="W128">
+        <v>0.5</v>
+      </c>
+      <c r="X128" t="str">
+        <v/>
+      </c>
+      <c r="Y128" t="str">
+        <v/>
+      </c>
+      <c r="Z128">
+        <v>-1</v>
+      </c>
+      <c r="AA128" t="str">
+        <v>dropbar/icon_type_6</v>
+      </c>
+      <c r="AB128" t="str">
+        <v/>
+      </c>
+      <c r="AC128" t="str">
+        <v/>
+      </c>
+      <c r="AD128">
+        <v>0</v>
+      </c>
+      <c r="AE128" t="str">
+        <v/>
+      </c>
+      <c r="AF128" t="str">
+        <v/>
+      </c>
+      <c r="AG128" t="str">
+        <v/>
+      </c>
+      <c r="AH128" t="str">
+        <v/>
+      </c>
+      <c r="AI128" t="str">
+        <v/>
+      </c>
+      <c r="AJ128">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129">
+        <v>1700104</v>
+      </c>
+      <c r="B129" t="str">
+        <v>华丽礼花</v>
+      </c>
+      <c r="C129" t="str">
+        <v/>
+      </c>
+      <c r="D129" t="str">
+        <v/>
+      </c>
+      <c r="E129" t="str">
+        <v>1</v>
+      </c>
+      <c r="F129" t="str">
+        <v>华丽礼花</v>
+      </c>
+      <c r="G129" t="str">
+        <v>zhuangbei/103/601</v>
+      </c>
+      <c r="H129" t="str">
+        <v/>
+      </c>
+      <c r="I129" t="str">
+        <v/>
+      </c>
+      <c r="J129" t="str">
+        <v/>
+      </c>
+      <c r="K129" t="str">
+        <v/>
+      </c>
+      <c r="L129" t="str">
+        <v/>
+      </c>
+      <c r="M129">
+        <v>4</v>
+      </c>
+      <c r="N129" t="str">
+        <v/>
+      </c>
+      <c r="O129" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P129">
+        <v>1</v>
+      </c>
+      <c r="Q129" t="str">
+        <v/>
+      </c>
+      <c r="R129">
+        <v>1</v>
+      </c>
+      <c r="S129" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T129" t="str">
+        <v/>
+      </c>
+      <c r="U129">
+        <v>9999</v>
+      </c>
+      <c r="V129">
+        <v>1</v>
+      </c>
+      <c r="W129">
+        <v>0.5</v>
+      </c>
+      <c r="X129" t="str">
+        <v/>
+      </c>
+      <c r="Y129" t="str">
+        <v/>
+      </c>
+      <c r="Z129">
+        <v>-1</v>
+      </c>
+      <c r="AA129" t="str">
+        <v>dropbar/icon_type_6</v>
+      </c>
+      <c r="AB129" t="str">
+        <v/>
+      </c>
+      <c r="AC129" t="str">
+        <v/>
+      </c>
+      <c r="AD129">
+        <v>0</v>
+      </c>
+      <c r="AE129" t="str">
+        <v/>
+      </c>
+      <c r="AF129" t="str">
+        <v/>
+      </c>
+      <c r="AG129" t="str">
+        <v/>
+      </c>
+      <c r="AH129" t="str">
+        <v/>
+      </c>
+      <c r="AI129" t="str">
+        <v/>
+      </c>
+      <c r="AJ129">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130">
+        <v>1800101</v>
+      </c>
+      <c r="B130" t="str">
+        <v>精铁耳环</v>
+      </c>
+      <c r="C130" t="str">
+        <v/>
+      </c>
+      <c r="D130" t="str">
+        <v/>
+      </c>
+      <c r="E130" t="str">
+        <v>1</v>
+      </c>
+      <c r="F130" t="str">
+        <v>精铁耳环</v>
+      </c>
+      <c r="G130" t="str">
+        <v>zhuangbei/101/701</v>
+      </c>
+      <c r="H130" t="str">
+        <v/>
+      </c>
+      <c r="I130" t="str">
+        <v/>
+      </c>
+      <c r="J130" t="str">
+        <v/>
+      </c>
+      <c r="K130" t="str">
+        <v/>
+      </c>
+      <c r="L130" t="str">
+        <v/>
+      </c>
+      <c r="M130">
+        <v>4</v>
+      </c>
+      <c r="N130" t="str">
+        <v/>
+      </c>
+      <c r="O130" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P130">
+        <v>1</v>
+      </c>
+      <c r="Q130" t="str">
+        <v/>
+      </c>
+      <c r="R130">
+        <v>1</v>
+      </c>
+      <c r="S130" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T130" t="str">
+        <v/>
+      </c>
+      <c r="U130">
+        <v>9999</v>
+      </c>
+      <c r="V130">
+        <v>1</v>
+      </c>
+      <c r="W130">
+        <v>0.5</v>
+      </c>
+      <c r="X130" t="str">
+        <v/>
+      </c>
+      <c r="Y130" t="str">
+        <v/>
+      </c>
+      <c r="Z130">
+        <v>-1</v>
+      </c>
+      <c r="AA130" t="str">
+        <v>dropbar/icon_type_7</v>
+      </c>
+      <c r="AB130" t="str">
+        <v/>
+      </c>
+      <c r="AC130" t="str">
+        <v/>
+      </c>
+      <c r="AD130">
+        <v>0</v>
+      </c>
+      <c r="AE130" t="str">
+        <v/>
+      </c>
+      <c r="AF130" t="str">
+        <v/>
+      </c>
+      <c r="AG130" t="str">
+        <v/>
+      </c>
+      <c r="AH130" t="str">
+        <v/>
+      </c>
+      <c r="AI130" t="str">
+        <v/>
+      </c>
+      <c r="AJ130">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131">
+        <v>1800102</v>
+      </c>
+      <c r="B131" t="str">
+        <v>宝石耳环</v>
+      </c>
+      <c r="C131" t="str">
+        <v/>
+      </c>
+      <c r="D131" t="str">
+        <v/>
+      </c>
+      <c r="E131" t="str">
+        <v>1</v>
+      </c>
+      <c r="F131" t="str">
+        <v>宝石耳环</v>
+      </c>
+      <c r="G131" t="str">
+        <v>zhuangbei/103/701</v>
+      </c>
+      <c r="H131" t="str">
+        <v/>
+      </c>
+      <c r="I131" t="str">
+        <v/>
+      </c>
+      <c r="J131" t="str">
+        <v/>
+      </c>
+      <c r="K131" t="str">
+        <v/>
+      </c>
+      <c r="L131" t="str">
+        <v/>
+      </c>
+      <c r="M131">
+        <v>4</v>
+      </c>
+      <c r="N131" t="str">
+        <v/>
+      </c>
+      <c r="O131" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P131">
+        <v>1</v>
+      </c>
+      <c r="Q131" t="str">
+        <v/>
+      </c>
+      <c r="R131">
+        <v>1</v>
+      </c>
+      <c r="S131" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T131" t="str">
+        <v/>
+      </c>
+      <c r="U131">
+        <v>9999</v>
+      </c>
+      <c r="V131">
+        <v>1</v>
+      </c>
+      <c r="W131">
+        <v>0.5</v>
+      </c>
+      <c r="X131" t="str">
+        <v/>
+      </c>
+      <c r="Y131" t="str">
+        <v/>
+      </c>
+      <c r="Z131">
+        <v>-1</v>
+      </c>
+      <c r="AA131" t="str">
+        <v>dropbar/icon_type_7</v>
+      </c>
+      <c r="AB131" t="str">
+        <v/>
+      </c>
+      <c r="AC131" t="str">
+        <v/>
+      </c>
+      <c r="AD131">
+        <v>0</v>
+      </c>
+      <c r="AE131" t="str">
+        <v/>
+      </c>
+      <c r="AF131" t="str">
+        <v/>
+      </c>
+      <c r="AG131" t="str">
+        <v/>
+      </c>
+      <c r="AH131" t="str">
+        <v/>
+      </c>
+      <c r="AI131" t="str">
+        <v/>
+      </c>
+      <c r="AJ131">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132">
+        <v>1800103</v>
+      </c>
+      <c r="B132" t="str">
+        <v>珠光耳环</v>
+      </c>
+      <c r="C132" t="str">
+        <v/>
+      </c>
+      <c r="D132" t="str">
+        <v/>
+      </c>
+      <c r="E132" t="str">
+        <v>1</v>
+      </c>
+      <c r="F132" t="str">
+        <v>珠光耳环</v>
+      </c>
+      <c r="G132" t="str">
+        <v>zhuangbei/103/701</v>
+      </c>
+      <c r="H132" t="str">
+        <v/>
+      </c>
+      <c r="I132" t="str">
+        <v/>
+      </c>
+      <c r="J132" t="str">
+        <v/>
+      </c>
+      <c r="K132" t="str">
+        <v/>
+      </c>
+      <c r="L132" t="str">
+        <v/>
+      </c>
+      <c r="M132">
+        <v>4</v>
+      </c>
+      <c r="N132" t="str">
+        <v/>
+      </c>
+      <c r="O132" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P132">
+        <v>1</v>
+      </c>
+      <c r="Q132" t="str">
+        <v/>
+      </c>
+      <c r="R132">
+        <v>1</v>
+      </c>
+      <c r="S132" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T132" t="str">
+        <v/>
+      </c>
+      <c r="U132">
+        <v>9999</v>
+      </c>
+      <c r="V132">
+        <v>1</v>
+      </c>
+      <c r="W132">
+        <v>0.5</v>
+      </c>
+      <c r="X132" t="str">
+        <v/>
+      </c>
+      <c r="Y132" t="str">
+        <v/>
+      </c>
+      <c r="Z132">
+        <v>-1</v>
+      </c>
+      <c r="AA132" t="str">
+        <v>dropbar/icon_type_7</v>
+      </c>
+      <c r="AB132" t="str">
+        <v/>
+      </c>
+      <c r="AC132" t="str">
+        <v/>
+      </c>
+      <c r="AD132">
+        <v>0</v>
+      </c>
+      <c r="AE132" t="str">
+        <v/>
+      </c>
+      <c r="AF132" t="str">
+        <v/>
+      </c>
+      <c r="AG132" t="str">
+        <v/>
+      </c>
+      <c r="AH132" t="str">
+        <v/>
+      </c>
+      <c r="AI132" t="str">
+        <v/>
+      </c>
+      <c r="AJ132">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133">
+        <v>1900101</v>
+      </c>
+      <c r="B133" t="str">
+        <v>精铁项链</v>
+      </c>
+      <c r="C133" t="str">
+        <v/>
+      </c>
+      <c r="D133" t="str">
+        <v/>
+      </c>
+      <c r="E133" t="str">
+        <v>1</v>
+      </c>
+      <c r="F133" t="str">
+        <v>精铁项链</v>
+      </c>
+      <c r="G133" t="str">
+        <v>zhuangbei/101/801</v>
+      </c>
+      <c r="H133" t="str">
+        <v/>
+      </c>
+      <c r="I133" t="str">
+        <v/>
+      </c>
+      <c r="J133" t="str">
+        <v/>
+      </c>
+      <c r="K133" t="str">
+        <v/>
+      </c>
+      <c r="L133" t="str">
+        <v/>
+      </c>
+      <c r="M133">
+        <v>4</v>
+      </c>
+      <c r="N133" t="str">
+        <v/>
+      </c>
+      <c r="O133" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P133">
+        <v>1</v>
+      </c>
+      <c r="Q133" t="str">
+        <v/>
+      </c>
+      <c r="R133">
+        <v>1</v>
+      </c>
+      <c r="S133" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T133" t="str">
+        <v/>
+      </c>
+      <c r="U133">
+        <v>9999</v>
+      </c>
+      <c r="V133">
+        <v>1</v>
+      </c>
+      <c r="W133">
+        <v>0.5</v>
+      </c>
+      <c r="X133" t="str">
+        <v/>
+      </c>
+      <c r="Y133" t="str">
+        <v/>
+      </c>
+      <c r="Z133">
+        <v>-1</v>
+      </c>
+      <c r="AA133" t="str">
+        <v>dropbar/icon_type_8</v>
+      </c>
+      <c r="AB133" t="str">
+        <v/>
+      </c>
+      <c r="AC133" t="str">
+        <v/>
+      </c>
+      <c r="AD133">
+        <v>0</v>
+      </c>
+      <c r="AE133" t="str">
+        <v/>
+      </c>
+      <c r="AF133" t="str">
+        <v/>
+      </c>
+      <c r="AG133" t="str">
+        <v/>
+      </c>
+      <c r="AH133" t="str">
+        <v/>
+      </c>
+      <c r="AI133" t="str">
+        <v/>
+      </c>
+      <c r="AJ133">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134">
+        <v>1900102</v>
+      </c>
+      <c r="B134" t="str">
+        <v>宝石项链</v>
+      </c>
+      <c r="C134" t="str">
+        <v/>
+      </c>
+      <c r="D134" t="str">
+        <v/>
+      </c>
+      <c r="E134" t="str">
+        <v>1</v>
+      </c>
+      <c r="F134" t="str">
+        <v>宝石项链</v>
+      </c>
+      <c r="G134" t="str">
+        <v>zhuangbei/103/801</v>
+      </c>
+      <c r="H134" t="str">
+        <v/>
+      </c>
+      <c r="I134" t="str">
+        <v/>
+      </c>
+      <c r="J134" t="str">
+        <v/>
+      </c>
+      <c r="K134" t="str">
+        <v/>
+      </c>
+      <c r="L134" t="str">
+        <v/>
+      </c>
+      <c r="M134">
+        <v>4</v>
+      </c>
+      <c r="N134" t="str">
+        <v/>
+      </c>
+      <c r="O134" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P134">
+        <v>1</v>
+      </c>
+      <c r="Q134" t="str">
+        <v/>
+      </c>
+      <c r="R134">
+        <v>1</v>
+      </c>
+      <c r="S134" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T134" t="str">
+        <v/>
+      </c>
+      <c r="U134">
+        <v>9999</v>
+      </c>
+      <c r="V134">
+        <v>1</v>
+      </c>
+      <c r="W134">
+        <v>0.5</v>
+      </c>
+      <c r="X134" t="str">
+        <v/>
+      </c>
+      <c r="Y134" t="str">
+        <v/>
+      </c>
+      <c r="Z134">
+        <v>-1</v>
+      </c>
+      <c r="AA134" t="str">
+        <v>dropbar/icon_type_8</v>
+      </c>
+      <c r="AB134" t="str">
+        <v/>
+      </c>
+      <c r="AC134" t="str">
+        <v/>
+      </c>
+      <c r="AD134">
+        <v>0</v>
+      </c>
+      <c r="AE134" t="str">
+        <v/>
+      </c>
+      <c r="AF134" t="str">
+        <v/>
+      </c>
+      <c r="AG134" t="str">
+        <v/>
+      </c>
+      <c r="AH134" t="str">
+        <v/>
+      </c>
+      <c r="AI134" t="str">
+        <v/>
+      </c>
+      <c r="AJ134">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135">
+        <v>1900103</v>
+      </c>
+      <c r="B135" t="str">
+        <v>翡翠项链</v>
+      </c>
+      <c r="C135" t="str">
+        <v/>
+      </c>
+      <c r="D135" t="str">
+        <v/>
+      </c>
+      <c r="E135" t="str">
+        <v>1</v>
+      </c>
+      <c r="F135" t="str">
+        <v>翡翠项链</v>
+      </c>
+      <c r="G135" t="str">
+        <v>zhuangbei/103/801</v>
+      </c>
+      <c r="H135" t="str">
+        <v/>
+      </c>
+      <c r="I135" t="str">
+        <v/>
+      </c>
+      <c r="J135" t="str">
+        <v/>
+      </c>
+      <c r="K135" t="str">
+        <v/>
+      </c>
+      <c r="L135" t="str">
+        <v/>
+      </c>
+      <c r="M135">
+        <v>4</v>
+      </c>
+      <c r="N135" t="str">
+        <v/>
+      </c>
+      <c r="O135" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P135">
+        <v>1</v>
+      </c>
+      <c r="Q135" t="str">
+        <v/>
+      </c>
+      <c r="R135">
+        <v>1</v>
+      </c>
+      <c r="S135" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T135" t="str">
+        <v/>
+      </c>
+      <c r="U135">
+        <v>9999</v>
+      </c>
+      <c r="V135">
+        <v>1</v>
+      </c>
+      <c r="W135">
+        <v>0.5</v>
+      </c>
+      <c r="X135" t="str">
+        <v/>
+      </c>
+      <c r="Y135" t="str">
+        <v/>
+      </c>
+      <c r="Z135">
+        <v>-1</v>
+      </c>
+      <c r="AA135" t="str">
+        <v>dropbar/icon_type_8</v>
+      </c>
+      <c r="AB135" t="str">
+        <v/>
+      </c>
+      <c r="AC135" t="str">
+        <v/>
+      </c>
+      <c r="AD135">
+        <v>0</v>
+      </c>
+      <c r="AE135" t="str">
+        <v/>
+      </c>
+      <c r="AF135" t="str">
+        <v/>
+      </c>
+      <c r="AG135" t="str">
+        <v/>
+      </c>
+      <c r="AH135" t="str">
+        <v/>
+      </c>
+      <c r="AI135" t="str">
+        <v/>
+      </c>
+      <c r="AJ135">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136">
+        <v>2000101</v>
+      </c>
+      <c r="B136" t="str">
+        <v>精铁戒指</v>
+      </c>
+      <c r="C136" t="str">
+        <v/>
+      </c>
+      <c r="D136" t="str">
+        <v/>
+      </c>
+      <c r="E136" t="str">
+        <v>1</v>
+      </c>
+      <c r="F136" t="str">
+        <v>精铁戒指</v>
+      </c>
+      <c r="G136" t="str">
+        <v>zhuangbei/101/901</v>
+      </c>
+      <c r="H136" t="str">
+        <v/>
+      </c>
+      <c r="I136" t="str">
+        <v/>
+      </c>
+      <c r="J136" t="str">
+        <v/>
+      </c>
+      <c r="K136" t="str">
+        <v/>
+      </c>
+      <c r="L136" t="str">
+        <v/>
+      </c>
+      <c r="M136">
+        <v>4</v>
+      </c>
+      <c r="N136" t="str">
+        <v/>
+      </c>
+      <c r="O136" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P136">
+        <v>1</v>
+      </c>
+      <c r="Q136" t="str">
+        <v/>
+      </c>
+      <c r="R136">
+        <v>1</v>
+      </c>
+      <c r="S136" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T136" t="str">
+        <v/>
+      </c>
+      <c r="U136">
+        <v>9999</v>
+      </c>
+      <c r="V136">
+        <v>1</v>
+      </c>
+      <c r="W136">
+        <v>0.5</v>
+      </c>
+      <c r="X136" t="str">
+        <v/>
+      </c>
+      <c r="Y136" t="str">
+        <v/>
+      </c>
+      <c r="Z136">
+        <v>-1</v>
+      </c>
+      <c r="AA136" t="str">
+        <v>dropbar/icon_type_9</v>
+      </c>
+      <c r="AB136" t="str">
+        <v/>
+      </c>
+      <c r="AC136" t="str">
+        <v/>
+      </c>
+      <c r="AD136">
+        <v>0</v>
+      </c>
+      <c r="AE136" t="str">
+        <v/>
+      </c>
+      <c r="AF136" t="str">
+        <v/>
+      </c>
+      <c r="AG136" t="str">
+        <v/>
+      </c>
+      <c r="AH136" t="str">
+        <v/>
+      </c>
+      <c r="AI136" t="str">
+        <v/>
+      </c>
+      <c r="AJ136">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137">
+        <v>2000102</v>
+      </c>
+      <c r="B137" t="str">
+        <v>护法戒指</v>
+      </c>
+      <c r="C137" t="str">
+        <v/>
+      </c>
+      <c r="D137" t="str">
+        <v/>
+      </c>
+      <c r="E137" t="str">
+        <v>1</v>
+      </c>
+      <c r="F137" t="str">
+        <v>护法戒指</v>
+      </c>
+      <c r="G137" t="str">
+        <v>zhuangbei/101/901</v>
+      </c>
+      <c r="H137" t="str">
+        <v/>
+      </c>
+      <c r="I137" t="str">
+        <v/>
+      </c>
+      <c r="J137" t="str">
+        <v/>
+      </c>
+      <c r="K137" t="str">
+        <v/>
+      </c>
+      <c r="L137" t="str">
+        <v/>
+      </c>
+      <c r="M137">
+        <v>4</v>
+      </c>
+      <c r="N137" t="str">
+        <v/>
+      </c>
+      <c r="O137" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P137">
+        <v>1</v>
+      </c>
+      <c r="Q137" t="str">
+        <v/>
+      </c>
+      <c r="R137">
+        <v>1</v>
+      </c>
+      <c r="S137" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T137" t="str">
+        <v/>
+      </c>
+      <c r="U137">
+        <v>9999</v>
+      </c>
+      <c r="V137">
+        <v>1</v>
+      </c>
+      <c r="W137">
+        <v>0.5</v>
+      </c>
+      <c r="X137" t="str">
+        <v/>
+      </c>
+      <c r="Y137" t="str">
+        <v/>
+      </c>
+      <c r="Z137">
+        <v>-1</v>
+      </c>
+      <c r="AA137" t="str">
+        <v>dropbar/icon_type_9</v>
+      </c>
+      <c r="AB137" t="str">
+        <v/>
+      </c>
+      <c r="AC137" t="str">
+        <v/>
+      </c>
+      <c r="AD137">
+        <v>0</v>
+      </c>
+      <c r="AE137" t="str">
+        <v/>
+      </c>
+      <c r="AF137" t="str">
+        <v/>
+      </c>
+      <c r="AG137" t="str">
+        <v/>
+      </c>
+      <c r="AH137" t="str">
+        <v/>
+      </c>
+      <c r="AI137" t="str">
+        <v/>
+      </c>
+      <c r="AJ137">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138">
+        <v>2000103</v>
+      </c>
+      <c r="B138" t="str">
+        <v>翡翠戒指</v>
+      </c>
+      <c r="C138" t="str">
+        <v/>
+      </c>
+      <c r="D138" t="str">
+        <v/>
+      </c>
+      <c r="E138" t="str">
+        <v>1</v>
+      </c>
+      <c r="F138" t="str">
+        <v>翡翠戒指</v>
+      </c>
+      <c r="G138" t="str">
+        <v>zhuangbei/101/901</v>
+      </c>
+      <c r="H138" t="str">
+        <v/>
+      </c>
+      <c r="I138" t="str">
+        <v/>
+      </c>
+      <c r="J138" t="str">
+        <v/>
+      </c>
+      <c r="K138" t="str">
+        <v/>
+      </c>
+      <c r="L138" t="str">
+        <v/>
+      </c>
+      <c r="M138">
+        <v>4</v>
+      </c>
+      <c r="N138" t="str">
+        <v/>
+      </c>
+      <c r="O138" t="str">
+        <v>装备</v>
+      </c>
+      <c r="P138">
+        <v>1</v>
+      </c>
+      <c r="Q138" t="str">
+        <v/>
+      </c>
+      <c r="R138">
+        <v>1</v>
+      </c>
+      <c r="S138" t="str">
+        <v>[[104,1]]</v>
+      </c>
+      <c r="T138" t="str">
+        <v/>
+      </c>
+      <c r="U138">
+        <v>9999</v>
+      </c>
+      <c r="V138">
+        <v>1</v>
+      </c>
+      <c r="W138">
+        <v>0.5</v>
+      </c>
+      <c r="X138" t="str">
+        <v/>
+      </c>
+      <c r="Y138" t="str">
+        <v/>
+      </c>
+      <c r="Z138">
+        <v>-1</v>
+      </c>
+      <c r="AA138" t="str">
+        <v>dropbar/icon_type_9</v>
+      </c>
+      <c r="AB138" t="str">
+        <v/>
+      </c>
+      <c r="AC138" t="str">
+        <v/>
+      </c>
+      <c r="AD138">
+        <v>0</v>
+      </c>
+      <c r="AE138" t="str">
+        <v/>
+      </c>
+      <c r="AF138" t="str">
+        <v/>
+      </c>
+      <c r="AG138" t="str">
+        <v/>
+      </c>
+      <c r="AH138" t="str">
+        <v/>
+      </c>
+      <c r="AI138" t="str">
+        <v/>
+      </c>
+      <c r="AJ138">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AJ97"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AJ138"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>